<commit_message>
Correct and complete 0all/0error daily monitoring files for 2026-09-23
The 9/23 all-source file uploaded on 9/23 turned out to be a partial
capture of source B only (35 rows). This replaces it with the full A
source (141 rows) and adds the complete B source (174 rows, of which
the previous 35-row file was a strict subset), matching the standard
two-source daily pattern.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017zeJVws1vWyy9Mcydj9ZHx
</commit_message>
<xml_diff>
--- a/daily-triage/data/0error20260923.xlsx
+++ b/daily-triage/data/0error20260923.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,27 +436,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>error_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>error_type</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>error</t>
         </is>
       </c>
     </row>
@@ -464,91 +469,121 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>69-欧盟理事会新闻头条-15</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" t="n">
         <v>20260923</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>00-联合国 UNECE-1958年协议状态-01</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.consilium.europa.eu/en/press/press-releases/</t>
+          <t>https://unece.org/transport/road-transport/status-1958-agreement-and-annexed-regulations</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>page_load_error</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page.wait_for_selector: Timeout 60000ms exceeded.
-Call log:
-  - waiting for locator(".gsc-excerpt-list") to be visible
-</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.goto: Timeout 120000ms exceeded.
+Call log:
+  - navigating to "https://unece.org/transport/road-transport/status-1958-agreement-and-annexed-regulations", waiting until "networkidle"
+</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>71-斯洛伐克法律汇编-01</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3" t="n">
         <v>20260923</v>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00-联合国-1958年协议附录——汽车安全条例-02</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.zakonypreludi.sk/zz/nove-predpisy</t>
+          <t>https://unece.org/transport/standards/transport/vehicle-regulations-wp29/addenda-1958-agreement-regulations-161-180</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HTTPError</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>403 Client Error: Forbidden for url: https://www.zakonypreludi.sk/zz/nove-predpisy</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.goto: Timeout 180000ms exceeded.
+Call log:
+  - navigating to "https://unece.org/transport/standards/transport/vehicle-regulations-wp29/addenda-1958-agreement-regulations-161-180", waiting until "networkidle"
+</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>73-乌克兰法律数据库-02</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4" t="n">
         <v>20260923</v>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00-联合国-即将举行的会议和活动-14</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://zakon.rada.gov.ua/laws/find/a?text=%D1%82%D1%80%D0%B0%D0%BD%D1%81%D0%BF%D0%BE%D1%80%D1%82%D0%BD%D0%B8%D1%85+%D0%B7%D0%B0%D1%81%D0%BE%D0%B1%D1%96%D0%B2&amp;textl=1&amp;bool=and</t>
+          <t>https://unece.org/info/events/unece-meetings-and-events</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>主程序异常</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page.goto: net::ERR_TIMED_OUT at https://zakon.rada.gov.ua/laws/find/a?text=%D1%82%D1%80%D0%B0%D0%BD%D1%81%D0%BF%D0%BE%D1%80%D1%82%D0%BD%D0%B8%D1%85+%D0%B7%D0%B0%D1%81%D0%BE%D0%B1%D1%96%D0%B2&amp;textl=1&amp;bool=and
-Call log:
-  - navigating to "https://zakon.rada.gov.ua/laws/find/a?text=%D1%82%D1%80%D0%B0%D0%BD%D1%81%D0%BF%D0%BE%D1%80%D1%82%D0%BD%D0%B8%D1%85+%D0%B7%D0%B0%D1%81%D0%BE%D0%B1%D1%96%D0%B2&amp;textl=1&amp;bool=and", waiting until "load"
-</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Message: session not created: cannot connect to chrome at 127.0.0.1:62204
+from session not created: This version of ChromeDriver only supports Chrome version 154
+Current browser version is 153.0.8010.52; For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#sessionnotcreatedexception
+Stacktrace:
+	undetected_chromedriver!GetHandleVerifier [0x17e0f03+4de3]
+	undetected_chromedriver!(No symbol) [0x16f51f4]
+	undetected_chromedriver!(No symbol) [0x152c270]
+	undetected_chromedriver!(No symbol) [0x1569572]
+	undetected_chromedriver!(No symbol) [0x156857c]
+	undetected_chromedriver!(No symbol) [0x155e775]
+	undetected_chromedriver!(No symbol) [0x155e596]
+	undetected_chromedriver!(No symbol) [0x15a6550]
+	undetected_chromedriver!(No symbol) [0x15a5d57]
+	undetected_chromedriver!(No symbol) [0x1599b16]
+	undetected_chromedriver!(No symbol) [0x156c13a]
+	undetected_chromedriver!(No symbol) [0x156ce14]
+	undetected_chromedriver!GetHandleVerifier [0x1c799f4+49d8d4]
+	undetected_chromedriver!GetHandleVerifier [0x1c9a15b+4be03b]
+	undetected_chromedriver!GetHandleVerifier [0x191c3f2+1402d2]
+	undetected_chromedriver!GetHandleVerifier [0x19246e3+1485c3]
+	undetected_chromedriver!(No symbol) [0x17035c8]
+	undetected_chromedriver!(No symbol) [0x16fe648]
+	undetected_chromedriver!(No symbol) [0x16fe7f5]
+	undetected_chromedriver!(No symbol) [0x16eab37]
+	KERNEL32!BaseThreadInitThunk [0x76de0619+19]
+	ntdll!RtlGetAppContainerNamedObjectPath [0x7723784d+ed]
+	ntdll!RtlGetAppContainerNamedObjectPath [0x7723781d+bd]
+</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -556,27 +591,33 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>76-英国法规库-02</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>20260923</v>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>000-全球-国家数字标准馆——标准快讯</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.legislation.gov.uk/primary+secondary/2026?title=vehicle&amp;sort=type</t>
+          <t>https://www.ndls.org.cn/news/index?type=1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>browser</t>
+          <t>Error</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Event loop is closed! Is Playwright already stopped?</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.ndls.org.cn/news/index?type=1
+Call log:
+  - navigating to "https://www.ndls.org.cn/news/index?type=1", waiting until "load"
+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -584,27 +625,33 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>80-巴基斯坦商务部文件-01</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>000-英联邦法律信息研究所-03</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.commerce.gov.pk/sros/</t>
+          <t>https://commonlii.org/cgi-bin/sinosrch.cgi?query=vehicle;mask_path=%20;method=title;meta=%2Fcommonlii;view=date;offset=0;collapse-level=0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>page_error</t>
+          <t>crawl_error</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>页面内容异常，可能被拦截或需要登录</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.wait_for_selector: Timeout 60000ms exceeded.
+Call log:
+  - waiting for locator("ol[start=\"1\"]") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -612,15 +659,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>83-哈萨克斯坦司法部法律信息研究所-03</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>000-大洋洲法律信息研究所-04</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://adilet.zan.kz/kaz/search/docs/ir=%7C2_033003%7C1_009&amp;sort_field=dt</t>
+          <t>https://classic.austlii.edu.au/cgi-bin/sinosrch.cgi?query=vehicle;results=50;submit=Search;mask_world=;mask_path=;callback=on;method=auto;meta=%2Fau;view=date;offset=0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -632,10 +681,11 @@
         <is>
           <t xml:space="preserve">Page.wait_for_selector: Timeout 60000ms exceeded.
 Call log:
-  - waiting for locator("div.gs_8") to be visible
-</t>
-        </is>
-      </c>
+  - waiting for locator("ol[start=\"1\"]") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -643,47 +693,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>86-吉尔吉斯斯坦司法部-01</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>11-埃及Egypt埃及投资和外贸部 - 法规和指示-02</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://cbd.minjust.gov.kg/search-docs/ru</t>
+          <t>https://goeic.gov.eg/en/laws-and-decisions/list/967</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>browser_error</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">BrowserType.launch: Target page, context or browser has been closed
-Browser logs:
-╔════════════════════════════════════════════════════════════════════════════════════════════════╗
-║ Looks like you launched a headed browser without having a XServer running.                     ║
-║ Set either 'headless: true' or use 'xvfb-run &lt;your-playwright-app&gt;' before running Playwright. ║
-║                                                                                                ║
-║ &lt;3 Playwright Team                                                                             ║
-╚════════════════════════════════════════════════════════════════════════════════════════════════╝
-Call log:
-  - &lt;launching&gt; /root/.cache/ms-playwright/chromium-1208/chrome-linux64/chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --no-sandbox --start-maximized --disable-blink-features=AutomationControlled --disable-extensions --disable-infobars --disable-popup-blocking --disable-notifications --disable-gpu --no-sandbox --disable-dev-shm-usage --user-agent=Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/112.0.0.0 Safari/537.36 --accept-language=zh-CN,zh;q=0.9,en;q=0.8 --user-data-dir=/tmp/playwright_chromiumdev_profile-elpsnf --remote-debugging-pipe --no-startup-window
-  - &lt;launched&gt; pid=817857
-  - [pid=817857][err] [817857:817857:0923/012406.736236:ERROR:ui/ozone/platform/x11/ozone_platform_x11.cc:256] Missing X server or $DISPLAY
-  - [pid=817857][err] [817857:817857:0923/012406.747501:ERROR:ui/aura/env.cc:246] The platform failed to initialize.  Exiting.
-  - [pid=817857] &lt;gracefully close start&gt;
-  - [pid=817857] &lt;kill&gt;
-  - [pid=817857] &lt;will force kill&gt;
-  - [pid=817857] &lt;process did exit: exitCode=1, signal=null&gt;
-  - [pid=817857] starting temporary directories cleanup
-  - [pid=817857] finished temporary directories cleanup
-  - [pid=817857] &lt;gracefully close end&gt;
-</t>
-        </is>
-      </c>
+          <t>所有URL都无法访问</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -691,47 +724,33 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>91-土耳其阿克谢希尔工商会公告-02</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2-美国交通部通知与规则制定文件-01</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://aksehirtso.org.tr/duyurular.html</t>
+          <t>https://www.transportation.gov/regulations/federal-register-documents?page=0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>主程序异常</t>
+          <t>crawl_error</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">BrowserType.launch: Target page, context or browser has been closed
-Browser logs:
-╔════════════════════════════════════════════════════════════════════════════════════════════════╗
-║ Looks like you launched a headed browser without having a XServer running.                     ║
-║ Set either 'headless: true' or use 'xvfb-run &lt;your-playwright-app&gt;' before running Playwright. ║
-║                                                                                                ║
-║ &lt;3 Playwright Team                                                                             ║
-╚════════════════════════════════════════════════════════════════════════════════════════════════╝
-Call log:
-  - &lt;launching&gt; /root/.cache/ms-playwright/chromium-1208/chrome-linux64/chrome --disable-field-trial-config --disable-background-networking --disable-background-timer-throttling --disable-backgrounding-occluded-windows --disable-back-forward-cache --disable-breakpad --disable-client-side-phishing-detection --disable-component-extensions-with-background-pages --disable-component-update --no-default-browser-check --disable-default-apps --disable-dev-shm-usage --disable-extensions --disable-features=AvoidUnnecessaryBeforeUnloadCheckSync,BoundaryEventDispatchTracksNodeRemoval,DestroyProfileOnBrowserClose,DialMediaRouteProvider,GlobalMediaControls,HttpsUpgrades,LensOverlay,MediaRouter,PaintHolding,ThirdPartyStoragePartitioning,Translate,AutoDeElevate,RenderDocument,OptimizationHints --enable-features=CDPScreenshotNewSurface --allow-pre-commit-input --disable-hang-monitor --disable-ipc-flooding-protection --disable-popup-blocking --disable-prompt-on-repost --disable-renderer-backgrounding --force-color-profile=srgb --metrics-recording-only --no-first-run --password-store=basic --use-mock-keychain --no-service-autorun --export-tagged-pdf --disable-search-engine-choice-screen --unsafely-disable-devtools-self-xss-warnings --edge-skip-compat-layer-relaunch --enable-automation --disable-infobars --disable-search-engine-choice-screen --disable-sync --enable-unsafe-swiftshader --no-sandbox --disable-blink-features=AutomationControlled --no-sandbox --disable-setuid-sandbox --disable-dev-shm-usage --disable-gpu --disable-web-security --allow-running-insecure-content --disable-features=IsolateOrigins,site-per-process --user-data-dir=/tmp/playwright_chromiumdev_profile-PwPu1d --remote-debugging-pipe --no-startup-window
-  - &lt;launched&gt; pid=818638
-  - [pid=818638][err] [818638:818638:0923/012856.060523:ERROR:ui/ozone/platform/x11/ozone_platform_x11.cc:256] Missing X server or $DISPLAY
-  - [pid=818638][err] [818638:818638:0923/012856.060685:ERROR:ui/aura/env.cc:246] The platform failed to initialize.  Exiting.
-  - [pid=818638] &lt;gracefully close start&gt;
-  - [pid=818638] &lt;kill&gt;
-  - [pid=818638] &lt;will force kill&gt;
-  - [pid=818638] &lt;process did exit: exitCode=1, signal=null&gt;
-  - [pid=818638] starting temporary directories cleanup
-  - [pid=818638] finished temporary directories cleanup
-  - [pid=818638] &lt;gracefully close end&gt;
-</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.wait_for_selector: Timeout 120000ms exceeded.
+Call log:
+  - waiting for locator(".table-responsive table tbody") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -739,27 +758,33 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>94-伊拉克电子法规库-02</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2-美国国会高级立法-03</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://iraqld.e-sjc-services.iq/legislations/search-legislation</t>
+          <t>https://www.congress.gov/quick-search/legislation?wordsPhrases=%E2%80%9Cvehicle%22%2C+%22automotive%22%2C+%22drive%22%2C+%22transport%22&amp;include=on&amp;wordVariants=on&amp;titles=on&amp;congressGroups%5B0%5D=0&amp;congresses%5B0%5D=all&amp;legislationNumbers=&amp;legislativeAction=&amp;sponsor=on&amp;cosponsor=on&amp;representative=&amp;senator=</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>captcha_block</t>
+          <t>crawl_error</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>网站需要人机验证或访问被拦截</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.wait_for_selector: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("ol.basic-search-results-lists") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -767,30 +792,33 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>94-伊拉克标准化与质量控制组织-03</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>20260923</v>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>23-新喀里多尼亚-国家出版物-01</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://iraqi-standards.org/</t>
+          <t>https://www.nouvelle-caledonie.gouv.fr/contenu/recherche/(searchtext)/v%C3%A9hicules/(change)/52397856?SearchText=v%C3%A9hicules</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>crawl_error</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page.goto: net::ERR_CERT_DATE_INVALID at https://iraqi-standards.org/
-Call log:
-  - navigating to "https://iraqi-standards.org/", waiting until "load"
-</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page.goto: net::ERR_HTTP2_PROTOCOL_ERROR at https://www.nouvelle-caledonie.gouv.fr/contenu/recherche/(searchtext)/v%C3%A9hicules/(change)/52397856?SearchText=v%C3%A9hicules
+Call log:
+  - navigating to "https://www.nouvelle-caledonie.gouv.fr/contenu/recherche/(searchtext)/v%C3%A9hicules/(change)/52397856?SearchText=v%C3%A9hicules", waiting until "domcontentloaded"
+</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -798,29 +826,480 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>96-以色列议会-02</t>
+          <t>20260923</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>20260923</t>
+          <t>38-巴拿马法律信息系统-01</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://main.knesset.gov.il/apps/legislation/main/laws?LawValidity=6079</t>
+          <t>https://infojuridica.procuraduria-admon.gob.pa/especifica.php</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>element_timeout</t>
+          <t>网址访问不了</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>等待页面元素超时，无法获取数据</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Locator.fill: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("input#tema")
+</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>40-玻利维亚官方公报-01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>http://gacetaoficialdebolivia.gob.bo/normas/busquedag1?q=veh%C3%ADculo</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page.goto: net::ERR_NAME_NOT_RESOLVED at https://www.gacetaoficialdebolivia.gob.bo/normas/busquedag1?q=vehiculo
+Call log:
+  - navigating to "https://www.gacetaoficialdebolivia.gob.bo/normas/busquedag1?q=vehiculo", waiting until "domcontentloaded"
+</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>45-萨尔瓦多立法议会-01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.asamblea.gob.sv/leyes-y-decretos/busqueda-decretos</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Locator.click: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("#busqueda-palabra-interes-wrapper input#busqueda-boton-buscar").first
+    - locator resolved to &lt;input type="submit" value="Buscar" class="btn btn-blue-al" id="busqueda-boton-buscar"/&gt;
+  - attempting click action
+    - scrolling into view if needed
+    - done scrolling
+    - forcing action
+    - performing click action
+    - click action done
+    - waiting for scheduled navigations to finish
+</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>5-危地马拉官方公报</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://legal.dca.gob.gt/GestionDocumento/BusquedaDocumento</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page.wait_for_selector: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("#busqueda") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>63-拉脱维亚共和国立法电子门户网站-01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://likumi.lv/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>程序错误</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Locator.click: Timeout 180000ms exceeded.
+Call log:
+  - waiting for locator("#searchForm button[type=\"submit\"]")
+    - locator resolved to &lt;button type="submit" value="submit" class="btn search fcw fwb fsl rfloat" onclick="event.preventDefault(); searchExpand.send();"&gt;…&lt;/button&gt;
+  - attempting click action
+    2 × waiting for element to be visible, enabled and stable
+      - element is visible, enabled and stable
+      - scrolling into view if needed
+      - done scrolling
+      - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+    - retrying click action
+    - waiting 20ms
+    - waiting for element to be visible, enabled and stable
+    - element is visible, enabled and stable
+    - scrolling into view if needed
+    - done scrolling
+    - &lt;div class="" tabindex="0" role="dialog" data-nosnippet="" id="cookiescript_injected" aria-label="Cookie consent dialog"&gt;…&lt;/div&gt; from &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; subtree intercepts pointer events
+  2 × retrying click action
+      - waiting 100ms
+      - waiting for element to be visible, enabled and stable
+      - element is visible, enabled and stable
+      - scrolling into view if needed
+      - done scrolling
+      - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+  84 × retrying click action
+       - waiting 500ms
+       - waiting for element to be visible, enabled and stable
+       - element is visible, enabled and stable
+       - scrolling into view if needed
+       - done scrolling
+       - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+     - retrying click action
+       - waiting 500ms
+       - waiting for element to be visible, enabled and stable
+       - element is visible, enabled and stable
+       - scrolling into view if needed
+       - done scrolling
+       - &lt;div class="" tabindex="0" role="dialog" data-nosnippet="" id="cookiescript_injected" aria-label="Cookie consent dialog"&gt;…&lt;/div&gt; from &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; subtree intercepts pointer events
+     - retrying click action
+       - waiting 500ms
+       - waiting for element to be visible, enabled and stable
+       - element is visible, enabled and stable
+       - scrolling into view if needed
+       - done scrolling
+       - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+     - retrying click action
+       - waiting 500ms
+       - waiting for element to be visible, enabled and stable
+       - element is visible, enabled and stable
+       - scrolling into view if needed
+       - done scrolling
+       - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+  - retrying click action
+    - waiting 500ms
+    - waiting for element to be visible, enabled and stable
+    - element is visible, enabled and stable
+    - scrolling into view if needed
+    - done scrolling
+    - &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; intercepts pointer events
+  - retrying click action
+    - waiting 500ms
+    - waiting for element to be visible, enabled and stable
+    - element is visible, enabled and stable
+    - scrolling into view if needed
+    - done scrolling
+    - &lt;div class="" tabindex="0" role="dialog" data-nosnippet="" id="cookiescript_injected" aria-label="Cookie consent dialog"&gt;…&lt;/div&gt; from &lt;div id="cookiescript_injected_wrapper" data-cs-id="cookiescript_injected"&gt;…&lt;/div&gt; subtree intercepts pointer events
+  - retrying click action
+    - waiting 500ms
+</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>66-罗马尼亚司法部立法门户网站-01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://legislatie.just.ro/Public/RezultateCautare</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>程序错误</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>67-摩尔多瓦国家道路运输局-01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://anta.gov.md/anunturi</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page.goto: net::ERR_CONNECTION_TIMED_OUT at https://anta.gov.md/anunturi
+Call log:
+  - navigating to "https://anta.gov.md/anunturi", waiting until "load"
+</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>67-摩尔多瓦共和国国家法律行为登记册-02</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.legis.md/cautare/getResults?document_status=0&amp;nr_doc=&amp;datepicker1=&amp;publication_status=+-+TOATE+-+&amp;nr=&amp;publish_date=&amp;search_type=2&amp;search_string=vehicule</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TimeoutError</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Locator.wait_for: Timeout 120000ms exceeded.
+Call log:
+  - waiting for locator("table.table.d1") to be visible
+    - waiting for" https://www.legis.md/cautare/getResults?document_status=0&amp;nr_doc=&amp;datepicker1=&amp;publication_status=+-+TOATE+-+&amp;nr=&amp;publish_date=&amp;search_type=2&amp;search_string=vehicule" navigation to finish...
+    - navigated to "https://www.legis.md/cautare/getResults?document_status=0&amp;nr_doc=&amp;datepicker1=&amp;publication_status=+-+TOATE+-+&amp;nr=&amp;publish_date=&amp;search_type=2&amp;search_string=vehicule"
+</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">错误: Page.wait_for_selector: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("input#select-code") to be visible
+</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/transparency/comitology-register/screen/documents</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">错误: Page.wait_for_selector: Timeout 30000ms exceeded.
+Call log:
+  - waiting for locator("input#select-code") to be visible
+</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>69-欧盟文件-机动车技术委员会-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>8-新西兰法规库NewZealand-01</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.legislation.govt.nz/items/?search_term=vehicle&amp;search_field=title&amp;search_term=vehicle&amp;per_page=20&amp;sort_by=most_recently_updated&amp;legislation_status=in_force&amp;sort_by=most_recently_updated&amp;per_page=20</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>robot_check</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>机器人验证超时</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>8-新西兰交通部NewZealand-02</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.nzta.govt.nz/about-us/public-consultation-hub/current-consultations</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>未找到 grid grid--list-view 容器</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>20260923</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>85-韩国-1-韩国汽车制造商协会-汽车日报</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.kama.or.kr/NewsController</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>网址访问不了</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page.goto: net::ERR_HTTP_RESPONSE_CODE_FAILURE at https://www.kama.or.kr/NewsController
+Call log:
+  - navigating to "https://www.kama.or.kr/NewsController", waiting until "networkidle"
+</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>